<commit_message>
Cleaned up docs folder
</commit_message>
<xml_diff>
--- a/docs/EchoPlay_Materialliste_250514.xlsx
+++ b/docs/EchoPlay_Materialliste_250514.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tomni\Documents\Schule-lokal\IMS\IP\ims.project.echoplay\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E06D61AB-BF14-4DF6-A8A6-C6DC01406F36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B351AD3-710B-4BB6-81DA-EC559BDFF1A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-195" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="51">
   <si>
     <t>Komponente</t>
   </si>
@@ -174,6 +174,21 @@
   </si>
   <si>
     <t>ESP32 Prozessor um alles zu rechnen</t>
+  </si>
+  <si>
+    <t>PRT-12795</t>
+  </si>
+  <si>
+    <t>1568-12795-ND</t>
+  </si>
+  <si>
+    <t>https://www.digikey.ch/de/products/detail/sparkfun-electronics/12795/5993860?s=N4IgTCBcDaIAoCUAqBaAjGA7ATgKwgF0BfIA</t>
+  </si>
+  <si>
+    <t>Jumper Kabel M-M 20 pack</t>
+  </si>
+  <si>
+    <t>Käbel um ESP mit Box zu verbinden</t>
   </si>
 </sst>
 </file>
@@ -543,11 +558,11 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.28515625" customWidth="1"/>
     <col min="3" max="3" width="12.42578125" customWidth="1"/>
     <col min="4" max="4" width="7.85546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="21.42578125" bestFit="1" customWidth="1"/>
@@ -791,24 +806,53 @@
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="3"/>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3"/>
-      <c r="G9" s="3"/>
+      <c r="A9" s="3">
+        <v>1</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="F9" t="s">
+        <v>46</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>48</v>
+      </c>
       <c r="H9" s="5">
-        <f>SUM(H2:H8)</f>
-        <v>63.74</v>
-      </c>
-      <c r="I9" s="3"/>
+        <v>2.3199999999999998</v>
+      </c>
+      <c r="I9" s="3" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="H10" s="1"/>
+      <c r="A10" s="3"/>
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="5">
+        <f>SUM(H2:H9)</f>
+        <v>66.06</v>
+      </c>
+      <c r="I10" s="3"/>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="G11" s="6"/>
+      <c r="H11" s="1"/>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="G12" s="6"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>